<commit_message>
Melhorias nas magias e anotações gerais
</commit_message>
<xml_diff>
--- a/data/grimoire_data.xlsx
+++ b/data/grimoire_data.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AC3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,6 +496,9 @@
       <c r="AB1" t="str">
         <v>moeda_platina</v>
       </c>
+      <c r="AC1" t="str">
+        <v>criatura_invocada_json</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -528,10 +531,10 @@
         <v>Clérigo</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="str">
-        <v>[{"classe":"Clérigo","nivel":1},{"classe":"Duskblade","nivel":1}]</v>
+        <v>[{"classe":"Clérigo","nivel":"3"}]</v>
       </c>
       <c r="F3" t="str">
         <v>Humano</v>
@@ -552,31 +555,31 @@
         <v>Médio</v>
       </c>
       <c r="L3" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M3">
         <v>10</v>
       </c>
       <c r="N3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="O3">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="P3">
         <v>10</v>
       </c>
       <c r="Q3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R3">
+        <v>21</v>
+      </c>
+      <c r="S3">
+        <v>24</v>
+      </c>
+      <c r="T3">
         <v>18</v>
-      </c>
-      <c r="S3">
-        <v>16</v>
-      </c>
-      <c r="T3">
-        <v>16</v>
       </c>
       <c r="U3" t="str">
         <v>Neutro e Bom</v>
@@ -591,21 +594,24 @@
         <v>7</v>
       </c>
       <c r="Y3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Z3">
-        <v>0</v>
+        <v>363</v>
       </c>
       <c r="AA3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AB3">
         <v>0</v>
       </c>
+      <c r="AC3" t="str">
+        <v>{"criatura":{"nome":"Lobo Celestial","tipo":"Animal (Celestial)","tamanho":"Médio","pv":13,"ca":14,"ataque":"+3 mordida","dano":"1d6+1","deslocamento":"15 m","habilidades":["Derrubar (For 13), Farejador"]},"pv_atual":13,"pv_max":13,"nivel_sm":2}</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -652,7 +658,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -854,16 +860,96 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Convocar Monstro II</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Conjuração</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Convoca uma criatura extraplanar de nível 2 ou inferior por 1 rodada/nível.</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Convocar Monstro I</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Conjuração</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Convoca uma criatura extraplanar de nível 1 para ajudar por 1 rodada/nível.</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Curar Ferimentos Moderados</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Conjuração</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Cura 2d8+1/nível de dano (máx +10).</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Curar Ferimentos Leves</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Conjuração</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Cura 1d8+1/nível de dano (máx +5).</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -924,7 +1010,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -958,7 +1044,7 @@
         <v>2</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -975,25 +1061,42 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
         <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1026,13 +1129,13 @@
         <v>luvas</v>
       </c>
       <c r="D2" t="str">
-        <v>Luva braba</v>
+        <v/>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Luvas</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -1046,7 +1149,7 @@
         <v>arma_principal</v>
       </c>
       <c r="D3" t="str">
-        <v>Espada brabaa</v>
+        <v>Crossbow</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -1055,89 +1158,39 @@
         <v>Arma Principal</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>armadura</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Breastplate</v>
+      </c>
+      <c r="E4" t="str">
+        <v>5 de bonus, Max 3 Dex, 15kg</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Armadura</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>nome</v>
-      </c>
-      <c r="C1" t="str">
-        <v>quantidade</v>
-      </c>
-      <c r="D1" t="str">
-        <v>peso</v>
-      </c>
-      <c r="E1" t="str">
-        <v>info</v>
-      </c>
-      <c r="F1" t="str">
-        <v>personagem_id</v>
-      </c>
-      <c r="G1" t="str">
-        <v>icone</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Poção de cura</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>0.2</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2" t="str">
-        <v>🍷</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Corda</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>0.2</v>
-      </c>
-      <c r="E3" t="str">
-        <v>30m</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3" t="str">
-        <v>⛏️</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1217,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1265,32 +1318,9 @@
         <v>[{"usado":false,"nota":""},{"usado":false,"nota":""},{"usado":false,"nota":""}]</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Arcane Channeling</v>
-      </c>
-      <c r="C3" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Duskblade</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3" t="str">
-        <v>[{"usado":false,"nota":""}]</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Talentos + Modal de anotações
</commit_message>
<xml_diff>
--- a/data/grimoire_data.xlsx
+++ b/data/grimoire_data.xlsx
@@ -497,7 +497,7 @@
         <v>moeda_platina</v>
       </c>
       <c r="AC1" t="str">
-        <v>criatura_invocada_json</v>
+        <v>bonus_slots_json</v>
       </c>
     </row>
     <row r="2">
@@ -594,10 +594,10 @@
         <v>7</v>
       </c>
       <c r="Y3">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="Z3">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="AA3">
         <v>4</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="AC3" t="str">
-        <v>{"criatura":{"nome":"Lobo Celestial","tipo":"Animal (Celestial)","tamanho":"Médio","pv":13,"ca":14,"ataque":"+3 mordida","dano":"1d6+1","deslocamento":"15 m","habilidades":["Derrubar (For 13), Farejador"]},"pv_atual":13,"pv_max":13,"nivel_sm":2}</v>
+        <v>[0,2,1,0,0,0,0,0,0,0]</v>
       </c>
     </row>
   </sheetData>
@@ -618,47 +618,231 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>titulo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>notas</v>
+      </c>
+      <c r="D1" t="str">
+        <v>personagem_id</v>
+      </c>
+      <c r="E1" t="str">
+        <v>data</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>A procura do acampamento orc</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Após a batalha do urso-coruja nós seguimos alguns rastros que encontramos no campo de batalha. Isso levou ao rastro de 2 orcs que enfrentamos e fizemos o possível para tirar informações em meio ao pantano humido e super dificil de se locomover.&lt;div&gt;&lt;br&gt;&lt;/div&gt;&lt;div&gt;Nós sequestramos o orc que sobreviver e torturamos para pegar algumas informações mas infelizmente não tivemos nenhum sucesso, por que durante o questionamento o orc tomou uma flechada nas costas de um grupo enorme de orcs que se aproximou ao nosso grupo.&lt;/div&gt;&lt;div&gt;&lt;br&gt;&lt;/div&gt;</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" t="str">
+        <v>09/04/2026</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nome</v>
+      </c>
+      <c r="C1" t="str">
+        <v>genero</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ocupacao</v>
+      </c>
+      <c r="E1" t="str">
+        <v>notas</v>
+      </c>
+      <c r="F1" t="str">
+        <v>foto_base64</v>
+      </c>
+      <c r="G1" t="str">
+        <v>personagem_id</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Dorn Escudo de coroa</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Masculino</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Encontramos anotações sobre ele no meio dos corpos que estavam no campo de batalha que enfrentamos o urso coruja próximo a melvont</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nome</v>
+      </c>
+      <c r="C1" t="str">
+        <v>notas</v>
+      </c>
+      <c r="D1" t="str">
+        <v>personagem_id</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Melvaunt</v>
+      </c>
+      <c r="C2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Uma cidade encontrada em uma ilha.
+Uma cidade diferente das outras, onde até escravidão é permitida, porem possui muita ordem.
+Controlada pela burguesia e grandes familias.
+Possui um mercado enorme com diversas mercadorias exoticas.</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nome</v>
+      </c>
+      <c r="C1" t="str">
+        <v>local_id</v>
+      </c>
+      <c r="D1" t="str">
+        <v>tipo</v>
+      </c>
+      <c r="E1" t="str">
+        <v>notas</v>
+      </c>
+      <c r="F1" t="str">
+        <v>npc_ids</v>
+      </c>
+      <c r="G1" t="str">
+        <v>personagem_id</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Sequestros de Melvaunt</v>
+      </c>
+      <c r="C2" t="str">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Principal</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Ao chegar Melvaunt para encontrar uma forma de ressucitar nosso companheiro Kush, nós descobrimos que a cidade estava passando por um momento dificil, pois filhos e membros das principais familias da nobreza estavam desaparecidos e estavam contratando aventureiros para encontrar o paradeiro dos nobres que sumiram.</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ressuscitar Kush</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>Secundária</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Infelizmente um dos nossos companheros faleceu durante a batalha no templo do sol e lua. Com isso o contruto Mitralhiam decidiu que nós iriamos achar alguma forma de ressuscitar o nosso companheiro.</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -940,16 +1124,36 @@
         <v>1</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Comando</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Encantamento</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Uma criatura obedece a um comando de uma palavra.</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1010,7 +1214,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1027,13 +1231,13 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1061,7 +1265,7 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1078,18 +1282,69 @@
         <v>2</v>
       </c>
       <c r="C8">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>11</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>12</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1207,10 +1462,115 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:F5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nome</v>
+      </c>
+      <c r="C1" t="str">
+        <v>classe</v>
+      </c>
+      <c r="D1" t="str">
+        <v>raca</v>
+      </c>
+      <c r="E1" t="str">
+        <v>notas</v>
+      </c>
+      <c r="F1" t="str">
+        <v>personagem_id</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Apollyon (Thales)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Hexblade</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Humano</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Completamente maluco das ideias.
+Ele se juntou ao nosso grupo por um suposto objetivo que temos em comum, mas eu não fui a fundo para descobrir qual é porque estamos em uma cidade que não conhecemos e quanto mais pessoas no grupo melhor.
+Durante a batalha com o urso coruja nós descobrimos que ele possui um problema com sangramento, onde ao acontecer um sangramento de alguém durante uma batalha, pode acontecer do Apollyon não resistir a tentaçao e ficar agressivo e completamente enlouquecido contra o alvo que está sofrendo o sangramento.</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>MITRALHIAM (Magnum)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Warbound</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Contruto</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Um construto bem literal. 
+Ele é um companheiro que vale a pena ter ao lado, apesar de não ter delicadesa com suas palvras, ele parece estar sempre tentando fazer o certo para chegar ao objetivo.</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Vonklad (Vitor)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Paladino</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Anão</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Um paladino da liberdade que está sempre procurando alguma confusão.
+Dito isso é importante mencionar que mesmo com o temperamento dificil ele parece ter bom coração e quer fazer o justo para manter a liberdade dos aliados e inimigos.</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cimérgia (Geicimar)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Duida</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Elfo</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Um druida gentil e muito esforçado. Mesmo com toda a sua timidez ele está sempre tando o seu máximo para ser útil par ao time com o dano avassalador de seu arco ou com suas magias de cura fenomenais.</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Contextos + Design System
</commit_message>
<xml_diff>
--- a/data/grimoire_data.xlsx
+++ b/data/grimoire_data.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AD3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -499,6 +499,9 @@
       <c r="AC1" t="str">
         <v>bonus_slots_json</v>
       </c>
+      <c r="AD1" t="str">
+        <v>criatura_invocada_json</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -611,7 +614,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -842,7 +845,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1144,9 +1147,49 @@
         <v>1</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Estabilizar</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Conjuração</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Estabiliza criatura que está morrendo.</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Purificar Comida e Água</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Transmutação</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Purifica comida e água podres.</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1214,7 +1257,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1231,13 +1274,13 @@
         <v>2</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1248,13 +1291,13 @@
         <v>2</v>
       </c>
       <c r="C6">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1265,7 +1308,7 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1282,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="C8">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1299,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="C9">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1322,7 +1365,7 @@
         <v>1</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1339,7 +1382,7 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>